<commit_message>
feat(tendo-brand): delivery-order 新增 xlsx→PDF 导出与签名叠加
- 生成 xlsx 后经 Excel COM 导出 PDF
- PyMuPDF 在 Requested By 签名区叠加 cailleach.png 签名图片
- G5 日期改为 datetime 对象 + 保留模板 number_format 渲染
- 长文本自动换行（wrap_text），地址行加高
- Submitted By 默认值改为 Cailleach.Zou
- 新增模板 TCMR2603-00005 与设计文档、实施计划、测试输出

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tendo-brand/test/TCMR2607-00010- Material Requisition - TCSO2607-00110.xlsx
+++ b/tendo-brand/test/TCMR2607-00010- Material Requisition - TCSO2607-00110.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Requisition" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,14 +17,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="[$-14809]d\ mmmm\,\ yyyy;@"/>
     <numFmt numFmtId="165" formatCode="_ [$¥-804]* #,##0.00_ ;_ [$¥-804]* \-#,##0.00_ ;_ [$¥-804]* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="166" formatCode="_ [$¥-804]* #,##0_ ;_ [$¥-804]* \-#,##0_ ;_ [$¥-804]* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="167" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="35">
     <font>
       <name val="Arial"/>
       <charset val="134"/>
@@ -71,17 +70,6 @@
     <font>
       <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color indexed="8"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
       <color indexed="4"/>
       <sz val="10"/>
       <u val="single"/>
@@ -273,12 +261,6 @@
       <sz val="12"/>
       <scheme val="major"/>
     </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <sz val="12"/>
-    </font>
   </fonts>
   <fills count="26">
     <fill>
@@ -289,7 +271,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.1499679555650502"/>
+        <fgColor theme="0" tint="-0.1499374370555742"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -432,7 +414,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="39">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -495,17 +477,6 @@
       <right style="thin">
         <color theme="1"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right/>
       <top/>
       <bottom style="thin">
         <color theme="1"/>
@@ -788,12 +759,36 @@
     </border>
     <border>
       <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
       <top style="thin">
         <color auto="1"/>
       </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -801,24 +796,9 @@
       <left/>
       <right/>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -831,28 +811,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color theme="1"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
       <top style="thin">
         <color theme="1"/>
       </top>
@@ -862,10 +833,10 @@
     <border>
       <left/>
       <right style="thin">
-        <color theme="1"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color theme="1"/>
+        <color auto="1"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -873,61 +844,61 @@
   </borders>
   <cellStyleXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="22" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="21"/>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="22"/>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="6" borderId="0"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="23"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="25"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="21"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="26"/>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="25" borderId="27"/>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="28"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="20"/>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="21"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="22"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="23"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="20"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25"/>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="29"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="26"/>
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="27"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="28"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -956,188 +927,170 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="7"/>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="52">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma 2" xfId="1"/>
     <cellStyle name="Currency 2" xfId="2"/>
     <cellStyle name="Hyperlink 2" xfId="3"/>
@@ -1191,7 +1144,74 @@
     <cellStyle name="Warning Text 2" xfId="51"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1412,22 +1432,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K51"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.69921875" defaultRowHeight="13.2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="12.45"/>
   <cols>
-    <col width="5.296875" customWidth="1" style="2" min="1" max="1"/>
-    <col width="20.8984375" customWidth="1" style="2" min="2" max="3"/>
-    <col width="38.59765625" customWidth="1" style="2" min="4" max="4"/>
-    <col width="25.296875" customWidth="1" style="2" min="5" max="5"/>
-    <col width="8.09765625" customWidth="1" style="2" min="6" max="6"/>
-    <col width="19.69921875" bestFit="1" customWidth="1" style="2" min="7" max="7"/>
-    <col width="18.59765625" customWidth="1" style="2" min="8" max="8"/>
-    <col width="13" customWidth="1" style="2" min="9" max="9"/>
-    <col width="13.296875" customWidth="1" style="2" min="10" max="11"/>
-    <col width="8.69921875" customWidth="1" style="2" min="12" max="16384"/>
+    <col width="5.28515625" customWidth="1" style="47" min="1" max="1"/>
+    <col width="20.92578125" customWidth="1" style="47" min="2" max="3"/>
+    <col width="38.5703125" customWidth="1" style="47" min="4" max="4"/>
+    <col width="25.28515625" customWidth="1" style="47" min="5" max="5"/>
+    <col width="8.0703125" customWidth="1" style="47" min="6" max="6"/>
+    <col width="19.7109375" bestFit="1" customWidth="1" style="47" min="7" max="7"/>
+    <col width="18.5703125" customWidth="1" style="47" min="8" max="8"/>
+    <col width="13" customWidth="1" style="47" min="9" max="9"/>
+    <col width="13.28515625" customWidth="1" style="47" min="10" max="11"/>
+    <col width="8.7109375" customWidth="1" style="47" min="12" max="12"/>
+    <col width="8.7109375" customWidth="1" style="47" min="13" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="44" t="inlineStr">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>Material Requisition</t>
         </is>
@@ -1461,7 +1482,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n"/>
-      <c r="C4" s="39" t="inlineStr"/>
+      <c r="C4" s="43" t="inlineStr"/>
       <c r="E4" s="13" t="inlineStr">
         <is>
           <t>Material Requisition No.</t>
@@ -1472,15 +1493,15 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G4" s="39" t="inlineStr">
+      <c r="G4" s="43" t="inlineStr">
         <is>
           <t>TCMR2607-00010</t>
         </is>
       </c>
-      <c r="H4" s="39" t="n"/>
-      <c r="I4" s="58" t="n"/>
-      <c r="J4" s="58" t="n"/>
-      <c r="K4" s="58" t="n"/>
+      <c r="H4" s="43" t="n"/>
+      <c r="I4" s="45" t="n"/>
+      <c r="J4" s="45" t="n"/>
+      <c r="K4" s="45" t="n"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
@@ -1489,7 +1510,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n"/>
-      <c r="C5" s="59" t="inlineStr">
+      <c r="C5" s="64" t="inlineStr">
         <is>
           <t>Cooley LLP Shanghai Representative Office</t>
         </is>
@@ -1504,24 +1525,22 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G5" s="60" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="H5" s="60" t="n"/>
+      <c r="G5" s="65" t="n">
+        <v>46225</v>
+      </c>
+      <c r="H5" s="65" t="n"/>
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="n"/>
       <c r="K5" s="7" t="n"/>
     </row>
-    <row r="6" ht="15.75" customFormat="1" customHeight="1" s="1">
+    <row r="6" ht="15.75" customFormat="1" customHeight="1" s="44">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Address:</t>
         </is>
       </c>
       <c r="B6" s="13" t="n"/>
-      <c r="C6" s="39" t="inlineStr">
+      <c r="C6" s="66" t="inlineStr">
         <is>
           <t>IFC - Tower 2 Level 35, Unit 3510, 8 Century Avenue, Pudong New Area, Shanghai, 200120</t>
         </is>
@@ -1536,23 +1555,23 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G6" s="39" t="inlineStr">
+      <c r="G6" s="43" t="inlineStr">
         <is>
           <t>CNY</t>
         </is>
       </c>
-      <c r="H6" s="39" t="n"/>
-      <c r="I6" s="58" t="n"/>
-      <c r="K6" s="58" t="n"/>
-    </row>
-    <row r="7" ht="15.75" customFormat="1" customHeight="1" s="1">
+      <c r="H6" s="43" t="n"/>
+      <c r="I6" s="45" t="n"/>
+      <c r="K6" s="45" t="n"/>
+    </row>
+    <row r="7" ht="15.75" customFormat="1" customHeight="1" s="44">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Sales Order No.:</t>
         </is>
       </c>
       <c r="B7" s="13" t="n"/>
-      <c r="C7" s="39" t="inlineStr">
+      <c r="C7" s="43" t="inlineStr">
         <is>
           <t>TCSO2607-00110</t>
         </is>
@@ -1567,22 +1586,22 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G7" s="61">
+      <c r="G7" s="67">
         <f>SUM(H12:H37)/1.13</f>
         <v/>
       </c>
-      <c r="H7" s="62" t="n"/>
-      <c r="I7" s="58" t="n"/>
-      <c r="K7" s="58" t="n"/>
-    </row>
-    <row r="8" ht="15.75" customFormat="1" customHeight="1" s="1">
+      <c r="H7" s="68" t="n"/>
+      <c r="I7" s="45" t="n"/>
+      <c r="K7" s="45" t="n"/>
+    </row>
+    <row r="8" ht="15.75" customFormat="1" customHeight="1" s="44">
       <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Sales Quotation No.:</t>
         </is>
       </c>
       <c r="B8" s="13" t="n"/>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="43" t="inlineStr">
         <is>
           <t>TCSQ2607-00184R2</t>
         </is>
@@ -1597,25 +1616,25 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G8" s="61">
+      <c r="G8" s="67">
         <f>G7*0.13</f>
         <v/>
       </c>
-      <c r="H8" s="61" t="n"/>
-      <c r="I8" s="58" t="n"/>
-      <c r="J8" s="58" t="n"/>
-      <c r="K8" s="58" t="n"/>
-    </row>
-    <row r="9" ht="15.75" customFormat="1" customHeight="1" s="1">
+      <c r="H8" s="67" t="n"/>
+      <c r="I8" s="45" t="n"/>
+      <c r="J8" s="45" t="n"/>
+      <c r="K8" s="45" t="n"/>
+    </row>
+    <row r="9" ht="15.75" customFormat="1" customHeight="1" s="44">
       <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Submitted By:</t>
         </is>
       </c>
       <c r="B9" s="28" t="n"/>
-      <c r="C9" s="39" t="inlineStr">
-        <is>
-          <t>Liu Shi Hao</t>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>Cailleach.Zou</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
@@ -1628,14 +1647,14 @@
           <t>:</t>
         </is>
       </c>
-      <c r="G9" s="61">
+      <c r="G9" s="67">
         <f>SUM(G7:G8)</f>
         <v/>
       </c>
-      <c r="H9" s="61" t="n"/>
-      <c r="I9" s="58" t="n"/>
-      <c r="J9" s="58" t="n"/>
-      <c r="K9" s="58" t="n"/>
+      <c r="H9" s="67" t="n"/>
+      <c r="I9" s="45" t="n"/>
+      <c r="J9" s="45" t="n"/>
+      <c r="K9" s="45" t="n"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="10" t="n"/>
@@ -1647,39 +1666,39 @@
       <c r="G10" s="10" t="n"/>
       <c r="H10" s="10" t="n"/>
     </row>
-    <row r="11" ht="15.6" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+    <row r="11" ht="15.65" customHeight="1">
+      <c r="A11" s="56" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="56" t="inlineStr">
         <is>
           <t>Part No.</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="56" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D11" s="63" t="n"/>
-      <c r="E11" s="42" t="inlineStr">
+      <c r="D11" s="57" t="n"/>
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="56" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="G11" s="56" t="inlineStr">
         <is>
           <t>Unit Cost</t>
         </is>
       </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="H11" s="56" t="inlineStr">
         <is>
           <t>Total Cost</t>
         </is>
@@ -1687,7 +1706,7 @@
       <c r="I11" s="8" t="n"/>
       <c r="J11" s="8" t="n"/>
     </row>
-    <row r="12" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="12" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A12" s="16" t="n">
         <v>1</v>
       </c>
@@ -1696,12 +1715,12 @@
           <t>760191940</t>
         </is>
       </c>
-      <c r="C12" s="64" t="inlineStr">
+      <c r="C12" s="69" t="inlineStr">
         <is>
           <t>Faceplate 2-Port, White</t>
         </is>
       </c>
-      <c r="D12" s="65" t="n"/>
+      <c r="D12" s="40" t="n"/>
       <c r="E12" s="23" t="n">
         <v>4</v>
       </c>
@@ -1710,10 +1729,10 @@
           <t>个</t>
         </is>
       </c>
-      <c r="G12" s="66" t="n">
+      <c r="G12" s="70" t="n">
         <v>10</v>
       </c>
-      <c r="H12" s="66">
+      <c r="H12" s="70">
         <f>E12*G12</f>
         <v/>
       </c>
@@ -1721,18 +1740,18 @@
       <c r="J12" s="8" t="n"/>
       <c r="K12" s="8" t="n"/>
     </row>
-    <row r="13" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="13" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A13" s="16">
         <f>A12+1</f>
         <v/>
       </c>
       <c r="B13" s="27" t="n"/>
-      <c r="C13" s="64" t="n"/>
-      <c r="D13" s="65" t="n"/>
+      <c r="C13" s="39" t="n"/>
+      <c r="D13" s="40" t="n"/>
       <c r="E13" s="23" t="n"/>
       <c r="F13" s="15" t="n"/>
-      <c r="G13" s="66" t="n"/>
-      <c r="H13" s="66">
+      <c r="G13" s="70" t="n"/>
+      <c r="H13" s="70">
         <f>E13*G13</f>
         <v/>
       </c>
@@ -1740,18 +1759,18 @@
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
     </row>
-    <row r="14" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="14" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A14" s="16">
         <f>A13+1</f>
         <v/>
       </c>
       <c r="B14" s="27" t="n"/>
-      <c r="C14" s="64" t="n"/>
-      <c r="D14" s="65" t="n"/>
+      <c r="C14" s="39" t="n"/>
+      <c r="D14" s="40" t="n"/>
       <c r="E14" s="23" t="n"/>
       <c r="F14" s="15" t="n"/>
-      <c r="G14" s="66" t="n"/>
-      <c r="H14" s="66">
+      <c r="G14" s="70" t="n"/>
+      <c r="H14" s="70">
         <f>E14*G14</f>
         <v/>
       </c>
@@ -1759,18 +1778,18 @@
       <c r="J14" s="8" t="n"/>
       <c r="K14" s="8" t="n"/>
     </row>
-    <row r="15" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="15" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A15" s="16">
         <f>A14+1</f>
         <v/>
       </c>
       <c r="B15" s="27" t="n"/>
-      <c r="C15" s="64" t="n"/>
-      <c r="D15" s="65" t="n"/>
+      <c r="C15" s="39" t="n"/>
+      <c r="D15" s="40" t="n"/>
       <c r="E15" s="23" t="n"/>
       <c r="F15" s="15" t="n"/>
-      <c r="G15" s="66" t="n"/>
-      <c r="H15" s="66">
+      <c r="G15" s="70" t="n"/>
+      <c r="H15" s="70">
         <f>E15*G15</f>
         <v/>
       </c>
@@ -1778,18 +1797,18 @@
       <c r="J15" s="8" t="n"/>
       <c r="K15" s="8" t="n"/>
     </row>
-    <row r="16" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="16" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A16" s="16">
         <f>A15+1</f>
         <v/>
       </c>
       <c r="B16" s="27" t="n"/>
-      <c r="C16" s="64" t="n"/>
-      <c r="D16" s="65" t="n"/>
+      <c r="C16" s="39" t="n"/>
+      <c r="D16" s="40" t="n"/>
       <c r="E16" s="23" t="n"/>
       <c r="F16" s="15" t="n"/>
-      <c r="G16" s="66" t="n"/>
-      <c r="H16" s="66">
+      <c r="G16" s="70" t="n"/>
+      <c r="H16" s="70">
         <f>E16*G16</f>
         <v/>
       </c>
@@ -1797,18 +1816,18 @@
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
     </row>
-    <row r="17" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="17" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A17" s="16">
         <f>A16+1</f>
         <v/>
       </c>
       <c r="B17" s="27" t="n"/>
-      <c r="C17" s="64" t="n"/>
-      <c r="D17" s="65" t="n"/>
+      <c r="C17" s="39" t="n"/>
+      <c r="D17" s="40" t="n"/>
       <c r="E17" s="23" t="n"/>
       <c r="F17" s="15" t="n"/>
-      <c r="G17" s="66" t="n"/>
-      <c r="H17" s="66">
+      <c r="G17" s="70" t="n"/>
+      <c r="H17" s="70">
         <f>E17*G17</f>
         <v/>
       </c>
@@ -1816,18 +1835,18 @@
       <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
     </row>
-    <row r="18" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="18" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A18" s="16">
         <f>A17+1</f>
         <v/>
       </c>
       <c r="B18" s="27" t="n"/>
-      <c r="C18" s="64" t="n"/>
-      <c r="D18" s="65" t="n"/>
+      <c r="C18" s="39" t="n"/>
+      <c r="D18" s="40" t="n"/>
       <c r="E18" s="23" t="n"/>
       <c r="F18" s="15" t="n"/>
-      <c r="G18" s="66" t="n"/>
-      <c r="H18" s="66">
+      <c r="G18" s="70" t="n"/>
+      <c r="H18" s="70">
         <f>E18*G18</f>
         <v/>
       </c>
@@ -1835,18 +1854,18 @@
       <c r="J18" s="8" t="n"/>
       <c r="K18" s="8" t="n"/>
     </row>
-    <row r="19" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="19" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A19" s="16">
         <f>A18+1</f>
         <v/>
       </c>
       <c r="B19" s="27" t="n"/>
-      <c r="C19" s="64" t="n"/>
-      <c r="D19" s="65" t="n"/>
+      <c r="C19" s="39" t="n"/>
+      <c r="D19" s="40" t="n"/>
       <c r="E19" s="23" t="n"/>
       <c r="F19" s="15" t="n"/>
-      <c r="G19" s="66" t="n"/>
-      <c r="H19" s="66">
+      <c r="G19" s="70" t="n"/>
+      <c r="H19" s="70">
         <f>E19*G19</f>
         <v/>
       </c>
@@ -1854,18 +1873,18 @@
       <c r="J19" s="8" t="n"/>
       <c r="K19" s="8" t="n"/>
     </row>
-    <row r="20" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="20" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A20" s="16">
         <f>A19+1</f>
         <v/>
       </c>
       <c r="B20" s="27" t="n"/>
-      <c r="C20" s="64" t="n"/>
-      <c r="D20" s="65" t="n"/>
+      <c r="C20" s="39" t="n"/>
+      <c r="D20" s="40" t="n"/>
       <c r="E20" s="23" t="n"/>
       <c r="F20" s="15" t="n"/>
-      <c r="G20" s="66" t="n"/>
-      <c r="H20" s="66">
+      <c r="G20" s="70" t="n"/>
+      <c r="H20" s="70">
         <f>E20*G20</f>
         <v/>
       </c>
@@ -1873,18 +1892,18 @@
       <c r="J20" s="8" t="n"/>
       <c r="K20" s="8" t="n"/>
     </row>
-    <row r="21" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="21" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A21" s="16">
         <f>A20+1</f>
         <v/>
       </c>
       <c r="B21" s="27" t="n"/>
-      <c r="C21" s="64" t="n"/>
-      <c r="D21" s="65" t="n"/>
+      <c r="C21" s="39" t="n"/>
+      <c r="D21" s="40" t="n"/>
       <c r="E21" s="23" t="n"/>
       <c r="F21" s="15" t="n"/>
-      <c r="G21" s="66" t="n"/>
-      <c r="H21" s="66">
+      <c r="G21" s="70" t="n"/>
+      <c r="H21" s="70">
         <f>E21*G21</f>
         <v/>
       </c>
@@ -1892,197 +1911,197 @@
       <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
     </row>
-    <row r="22" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="22" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A22" s="16" t="n"/>
       <c r="B22" s="27" t="n"/>
-      <c r="C22" s="64" t="n"/>
-      <c r="D22" s="65" t="n"/>
+      <c r="C22" s="39" t="n"/>
+      <c r="D22" s="40" t="n"/>
       <c r="E22" s="23" t="n"/>
       <c r="F22" s="15" t="n"/>
-      <c r="G22" s="66" t="n"/>
-      <c r="H22" s="66" t="n"/>
+      <c r="G22" s="70" t="n"/>
+      <c r="H22" s="70" t="n"/>
       <c r="I22" s="8" t="n"/>
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
     </row>
-    <row r="23" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="23" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A23" s="16" t="n"/>
       <c r="B23" s="27" t="n"/>
-      <c r="C23" s="64" t="n"/>
-      <c r="D23" s="65" t="n"/>
+      <c r="C23" s="39" t="n"/>
+      <c r="D23" s="40" t="n"/>
       <c r="E23" s="23" t="n"/>
       <c r="F23" s="15" t="n"/>
-      <c r="G23" s="66" t="n"/>
-      <c r="H23" s="66" t="n"/>
+      <c r="G23" s="70" t="n"/>
+      <c r="H23" s="70" t="n"/>
       <c r="I23" s="8" t="n"/>
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
     </row>
-    <row r="24" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="24" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A24" s="16" t="n"/>
       <c r="B24" s="27" t="n"/>
-      <c r="C24" s="64" t="n"/>
-      <c r="D24" s="65" t="n"/>
+      <c r="C24" s="39" t="n"/>
+      <c r="D24" s="40" t="n"/>
       <c r="E24" s="23" t="n"/>
       <c r="F24" s="15" t="n"/>
-      <c r="G24" s="66" t="n"/>
-      <c r="H24" s="66" t="n"/>
+      <c r="G24" s="70" t="n"/>
+      <c r="H24" s="70" t="n"/>
       <c r="I24" s="8" t="n"/>
       <c r="J24" s="8" t="n"/>
       <c r="K24" s="8" t="n"/>
     </row>
-    <row r="25" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="25" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A25" s="16" t="n"/>
       <c r="B25" s="27" t="n"/>
-      <c r="C25" s="64" t="n"/>
-      <c r="D25" s="65" t="n"/>
+      <c r="C25" s="39" t="n"/>
+      <c r="D25" s="40" t="n"/>
       <c r="E25" s="23" t="n"/>
       <c r="F25" s="15" t="n"/>
-      <c r="G25" s="66" t="n"/>
-      <c r="H25" s="66" t="n"/>
+      <c r="G25" s="70" t="n"/>
+      <c r="H25" s="70" t="n"/>
       <c r="I25" s="8" t="n"/>
       <c r="J25" s="8" t="n"/>
       <c r="K25" s="8" t="n"/>
     </row>
-    <row r="26" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="26" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A26" s="16" t="n"/>
       <c r="B26" s="27" t="n"/>
-      <c r="C26" s="64" t="n"/>
-      <c r="D26" s="65" t="n"/>
+      <c r="C26" s="39" t="n"/>
+      <c r="D26" s="40" t="n"/>
       <c r="E26" s="23" t="n"/>
       <c r="F26" s="15" t="n"/>
-      <c r="G26" s="66" t="n"/>
-      <c r="H26" s="66" t="n"/>
+      <c r="G26" s="70" t="n"/>
+      <c r="H26" s="70" t="n"/>
       <c r="I26" s="8" t="n"/>
       <c r="J26" s="8" t="n"/>
       <c r="K26" s="8" t="n"/>
     </row>
-    <row r="27" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="27" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A27" s="16" t="n"/>
       <c r="B27" s="27" t="n"/>
-      <c r="C27" s="64" t="n"/>
-      <c r="D27" s="65" t="n"/>
+      <c r="C27" s="39" t="n"/>
+      <c r="D27" s="40" t="n"/>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="15" t="n"/>
-      <c r="G27" s="66" t="n"/>
-      <c r="H27" s="66" t="n"/>
+      <c r="G27" s="70" t="n"/>
+      <c r="H27" s="70" t="n"/>
       <c r="I27" s="8" t="n"/>
       <c r="J27" s="8" t="n"/>
       <c r="K27" s="8" t="n"/>
     </row>
-    <row r="28" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="28" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A28" s="16" t="n"/>
       <c r="B28" s="27" t="n"/>
-      <c r="C28" s="64" t="n"/>
-      <c r="D28" s="65" t="n"/>
+      <c r="C28" s="39" t="n"/>
+      <c r="D28" s="40" t="n"/>
       <c r="E28" s="23" t="n"/>
       <c r="F28" s="15" t="n"/>
-      <c r="G28" s="66" t="n"/>
-      <c r="H28" s="66" t="n"/>
+      <c r="G28" s="70" t="n"/>
+      <c r="H28" s="70" t="n"/>
       <c r="I28" s="8" t="n"/>
       <c r="J28" s="8" t="n"/>
       <c r="K28" s="8" t="n"/>
     </row>
-    <row r="29" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="29" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A29" s="16" t="n"/>
       <c r="B29" s="27" t="n"/>
-      <c r="C29" s="64" t="n"/>
-      <c r="D29" s="65" t="n"/>
+      <c r="C29" s="39" t="n"/>
+      <c r="D29" s="40" t="n"/>
       <c r="E29" s="23" t="n"/>
       <c r="F29" s="15" t="n"/>
-      <c r="G29" s="66" t="n"/>
-      <c r="H29" s="66" t="n"/>
+      <c r="G29" s="70" t="n"/>
+      <c r="H29" s="70" t="n"/>
       <c r="I29" s="8" t="n"/>
       <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
     </row>
-    <row r="30" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="30" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A30" s="16" t="n"/>
       <c r="B30" s="27" t="n"/>
-      <c r="C30" s="64" t="n"/>
-      <c r="D30" s="65" t="n"/>
+      <c r="C30" s="39" t="n"/>
+      <c r="D30" s="40" t="n"/>
       <c r="E30" s="23" t="n"/>
       <c r="F30" s="15" t="n"/>
-      <c r="G30" s="66" t="n"/>
-      <c r="H30" s="66" t="n"/>
+      <c r="G30" s="70" t="n"/>
+      <c r="H30" s="70" t="n"/>
       <c r="I30" s="8" t="n"/>
       <c r="J30" s="8" t="n"/>
       <c r="K30" s="8" t="n"/>
     </row>
-    <row r="31" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="31" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A31" s="16" t="n"/>
       <c r="B31" s="27" t="n"/>
-      <c r="C31" s="64" t="n"/>
-      <c r="D31" s="65" t="n"/>
+      <c r="C31" s="39" t="n"/>
+      <c r="D31" s="40" t="n"/>
       <c r="E31" s="23" t="n"/>
       <c r="F31" s="15" t="n"/>
-      <c r="G31" s="66" t="n"/>
-      <c r="H31" s="66" t="n"/>
+      <c r="G31" s="70" t="n"/>
+      <c r="H31" s="70" t="n"/>
       <c r="I31" s="8" t="n"/>
       <c r="J31" s="8" t="n"/>
       <c r="K31" s="8" t="n"/>
     </row>
-    <row r="32" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="32" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A32" s="16" t="n"/>
       <c r="B32" s="27" t="n"/>
-      <c r="C32" s="64" t="n"/>
-      <c r="D32" s="65" t="n"/>
+      <c r="C32" s="39" t="n"/>
+      <c r="D32" s="40" t="n"/>
       <c r="E32" s="23" t="n"/>
       <c r="F32" s="15" t="n"/>
-      <c r="G32" s="66" t="n"/>
-      <c r="H32" s="66" t="n"/>
+      <c r="G32" s="70" t="n"/>
+      <c r="H32" s="70" t="n"/>
       <c r="I32" s="8" t="n"/>
       <c r="J32" s="8" t="n"/>
       <c r="K32" s="8" t="n"/>
     </row>
-    <row r="33" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="33" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A33" s="16" t="n"/>
       <c r="B33" s="27" t="n"/>
-      <c r="C33" s="64" t="n"/>
-      <c r="D33" s="65" t="n"/>
+      <c r="C33" s="39" t="n"/>
+      <c r="D33" s="40" t="n"/>
       <c r="E33" s="23" t="n"/>
       <c r="F33" s="15" t="n"/>
-      <c r="G33" s="66" t="n"/>
-      <c r="H33" s="66" t="n"/>
+      <c r="G33" s="70" t="n"/>
+      <c r="H33" s="70" t="n"/>
       <c r="I33" s="8" t="n"/>
       <c r="J33" s="8" t="n"/>
       <c r="K33" s="8" t="n"/>
     </row>
-    <row r="34" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="34" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A34" s="16" t="n"/>
       <c r="B34" s="27" t="n"/>
-      <c r="C34" s="64" t="n"/>
-      <c r="D34" s="65" t="n"/>
+      <c r="C34" s="39" t="n"/>
+      <c r="D34" s="40" t="n"/>
       <c r="E34" s="23" t="n"/>
       <c r="F34" s="15" t="n"/>
-      <c r="G34" s="66" t="n"/>
-      <c r="H34" s="66" t="n"/>
+      <c r="G34" s="70" t="n"/>
+      <c r="H34" s="70" t="n"/>
       <c r="I34" s="8" t="n"/>
       <c r="J34" s="8" t="n"/>
       <c r="K34" s="8" t="n"/>
     </row>
-    <row r="35" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="35" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A35" s="16" t="n"/>
       <c r="B35" s="27" t="n"/>
-      <c r="C35" s="64" t="n"/>
-      <c r="D35" s="65" t="n"/>
+      <c r="C35" s="39" t="n"/>
+      <c r="D35" s="40" t="n"/>
       <c r="E35" s="23" t="n"/>
       <c r="F35" s="15" t="n"/>
-      <c r="G35" s="66" t="n"/>
-      <c r="H35" s="66" t="n"/>
+      <c r="G35" s="70" t="n"/>
+      <c r="H35" s="70" t="n"/>
       <c r="I35" s="8" t="n"/>
       <c r="J35" s="8" t="n"/>
       <c r="K35" s="8" t="n"/>
     </row>
-    <row r="36" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="36" ht="15" customFormat="1" customHeight="1" s="44">
       <c r="A36" s="16" t="n"/>
       <c r="B36" s="27" t="n"/>
-      <c r="C36" s="64" t="n"/>
-      <c r="D36" s="65" t="n"/>
+      <c r="C36" s="39" t="n"/>
+      <c r="D36" s="40" t="n"/>
       <c r="E36" s="23" t="n"/>
       <c r="F36" s="15" t="n"/>
-      <c r="G36" s="66" t="n"/>
-      <c r="H36" s="66" t="n"/>
+      <c r="G36" s="70" t="n"/>
+      <c r="H36" s="70" t="n"/>
       <c r="I36" s="8" t="n"/>
       <c r="J36" s="8" t="n"/>
       <c r="K36" s="8" t="n"/>
@@ -2090,8 +2109,8 @@
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="20" t="n"/>
       <c r="B37" s="20" t="n"/>
-      <c r="C37" s="67" t="n"/>
-      <c r="D37" s="68" t="n"/>
+      <c r="C37" s="62" t="n"/>
+      <c r="D37" s="63" t="n"/>
       <c r="E37" s="24" t="n"/>
       <c r="F37" s="37" t="n"/>
       <c r="G37" s="21" t="n"/>
@@ -2114,27 +2133,27 @@
       <c r="K38" s="8" t="n"/>
     </row>
     <row r="39" ht="31.5" customHeight="1">
-      <c r="A39" s="49" t="inlineStr">
+      <c r="A39" s="53" t="inlineStr">
         <is>
           <t>By signing below, the Employee acknowledged that the above materials had been withdraw.</t>
         </is>
       </c>
-      <c r="B39" s="69" t="n"/>
-      <c r="C39" s="69" t="n"/>
-      <c r="D39" s="70" t="n"/>
+      <c r="B39" s="54" t="n"/>
+      <c r="C39" s="54" t="n"/>
+      <c r="D39" s="55" t="n"/>
       <c r="E39" s="29" t="n"/>
       <c r="F39" s="29" t="n"/>
       <c r="G39" s="29" t="n"/>
       <c r="H39" s="29" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="49" t="inlineStr">
+      <c r="A40" s="53" t="inlineStr">
         <is>
           <t>Requested By:</t>
         </is>
       </c>
-      <c r="B40" s="69" t="n"/>
-      <c r="C40" s="70" t="n"/>
+      <c r="B40" s="54" t="n"/>
+      <c r="C40" s="55" t="n"/>
       <c r="D40" s="33" t="inlineStr">
         <is>
           <t>Approved By:</t>
@@ -2147,13 +2166,13 @@
       <c r="I40" s="26" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="54" t="inlineStr">
+      <c r="A41" s="41" t="inlineStr">
         <is>
           <t>Signature:</t>
         </is>
       </c>
-      <c r="B41" s="71" t="n"/>
-      <c r="C41" s="71" t="n"/>
+      <c r="B41" s="42" t="n"/>
+      <c r="C41" s="42" t="n"/>
       <c r="D41" s="30" t="inlineStr">
         <is>
           <t>Signature:</t>
@@ -2165,63 +2184,63 @@
       <c r="H41" s="26" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="72" t="n"/>
-      <c r="C42" s="73" t="n"/>
-      <c r="D42" s="50" t="n"/>
+      <c r="A42" s="48" t="n"/>
+      <c r="C42" s="49" t="n"/>
+      <c r="D42" s="60" t="n"/>
       <c r="E42" s="26" t="n"/>
       <c r="F42" s="26" t="n"/>
       <c r="G42" s="26" t="n"/>
       <c r="H42" s="26" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="74" t="n"/>
-      <c r="C43" s="73" t="n"/>
-      <c r="D43" s="75" t="n"/>
+      <c r="A43" s="50" t="n"/>
+      <c r="C43" s="49" t="n"/>
+      <c r="D43" s="61" t="n"/>
       <c r="E43" s="26" t="n"/>
       <c r="F43" s="26" t="n"/>
       <c r="G43" s="26" t="n"/>
       <c r="H43" s="26" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="74" t="n"/>
-      <c r="C44" s="73" t="n"/>
-      <c r="D44" s="75" t="n"/>
+      <c r="A44" s="50" t="n"/>
+      <c r="C44" s="49" t="n"/>
+      <c r="D44" s="61" t="n"/>
       <c r="E44" s="26" t="n"/>
       <c r="F44" s="26" t="n"/>
       <c r="G44" s="26" t="n"/>
       <c r="H44" s="26" t="n"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="74" t="n"/>
-      <c r="C45" s="73" t="n"/>
-      <c r="D45" s="75" t="n"/>
+      <c r="A45" s="50" t="n"/>
+      <c r="C45" s="49" t="n"/>
+      <c r="D45" s="61" t="n"/>
       <c r="E45" s="26" t="n"/>
       <c r="F45" s="26" t="n"/>
       <c r="G45" s="26" t="n"/>
       <c r="H45" s="26" t="n"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="74" t="n"/>
-      <c r="C46" s="73" t="n"/>
-      <c r="D46" s="75" t="n"/>
+      <c r="A46" s="50" t="n"/>
+      <c r="C46" s="49" t="n"/>
+      <c r="D46" s="61" t="n"/>
       <c r="E46" s="26" t="n"/>
       <c r="F46" s="26" t="n"/>
       <c r="G46" s="26" t="n"/>
       <c r="H46" s="26" t="n"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="74" t="n"/>
-      <c r="C47" s="73" t="n"/>
-      <c r="D47" s="75" t="n"/>
+      <c r="A47" s="50" t="n"/>
+      <c r="C47" s="49" t="n"/>
+      <c r="D47" s="61" t="n"/>
       <c r="E47" s="26" t="n"/>
       <c r="F47" s="26" t="n"/>
       <c r="G47" s="26" t="n"/>
       <c r="H47" s="26" t="n"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="45" t="inlineStr">
-        <is>
-          <t>Name:</t>
+      <c r="A48" s="59" t="inlineStr">
+        <is>
+          <t>Name:Cailleach Zou</t>
         </is>
       </c>
       <c r="D48" s="31" t="inlineStr">
@@ -2235,9 +2254,9 @@
       <c r="H48" s="26" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="45" t="inlineStr">
-        <is>
-          <t>Title:</t>
+      <c r="A49" s="59" t="inlineStr">
+        <is>
+          <t>Title:Senior Project Engineer</t>
         </is>
       </c>
       <c r="D49" s="31" t="inlineStr">
@@ -2251,13 +2270,13 @@
       <c r="H49" s="26" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="47" t="inlineStr">
-        <is>
-          <t>Date:</t>
-        </is>
-      </c>
-      <c r="B50" s="76" t="n"/>
-      <c r="C50" s="76" t="n"/>
+      <c r="A50" s="51" t="inlineStr">
+        <is>
+          <t>Date:22/07/26</t>
+        </is>
+      </c>
+      <c r="B50" s="52" t="n"/>
+      <c r="C50" s="52" t="n"/>
       <c r="D50" s="32" t="inlineStr">
         <is>
           <t>Date:</t>
@@ -2283,8 +2302,8 @@
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="C24:D24"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="C33:D33"/>
@@ -2311,14 +2330,14 @@
     <mergeCell ref="A40:C40"/>
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="A1:H2"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C23:D23"/>
     <mergeCell ref="A48:C48"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C17:D17"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="D42:D47"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="A49:C49"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C32:D32"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="C28:D28"/>
@@ -2326,7 +2345,7 @@
     <mergeCell ref="C18:D18"/>
   </mergeCells>
   <pageMargins left="0.5118110236220472" right="0.5118110236220472" top="0.8661417322834646" bottom="0.7086614173228347" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="53"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="54"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;G</oddHeader>
     <oddFooter>&amp;C&amp;12 Tendo Technology (Shanghai) Co., Ltd._x000a_Building B, Unit 206, No. 135 Yanping Road, Jingan District, Shanghai_x000a_腾都创迎（上海）科技有限公司_x000a_上海市静安区延平路135号B座206室&amp;R&amp;12 &amp;P</oddFooter>

</xml_diff>